<commit_message>
Correção das heurísticas não encontradas pela validação
</commit_message>
<xml_diff>
--- a/resources/filtered_papers_vulnerabilidades_2026.xlsx
+++ b/resources/filtered_papers_vulnerabilidades_2026.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -473,44 +473,44 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>conf/kbse/CeccatoNAB16</t>
+          <t>conf/icde/MengZK18</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>conf/kbse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Mariano Ceccato and Cu D. Nguyen and Dennis Appelt and Lionel C. Briand</t>
+          <t>Xianrui Meng and Haohan Zhu and George Kollios</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>SOFIA: an automated security oracle for black-box testing of SQL-injection vulnerabilities</t>
+          <t>Top-k Query Processing on Encrypted Databases with Strong Security Guarantees</t>
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2016</v>
+        <v>2018</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>conf/kbse/2016</t>
+          <t>conf/icde/2018</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>db/conf/kbse/ase2016.html#CeccatoNAB16</t>
+          <t>db/conf/icde/icde2018.html#MengZK18</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>@inproceedings{ceccato:2016,
-booktitle = {International Conference on Automated Software Engineering(ASE)}, 
-author = {Mariano Ceccato and Cu D. Nguyen and Dennis Appelt and Lionel C. Briand}, 
-title = {{SOFIA: an automated security oracle for black-box testing of SQL-injection vulnerabilities}}, 
-year = {2016} 
+          <t>@inproceedings{meng:2018,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Xianrui Meng and Haohan Zhu and George Kollios}, 
+title = {{Top-k Query Processing on Encrypted Databases with Strong Security Guarantees}}, 
+year = {2018} 
 }</t>
         </is>
       </c>
@@ -518,44 +518,44 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>conf/kbse/LiX0WZ24</t>
+          <t>conf/icde/Palley86</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>conf/kbse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Yuanlin Li and Zhiwei Xu and Min Zhou 0001 and Hai Wan and Xibin Zhao</t>
+          <t>Michael A. Palley</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Trident: Detecting SQL Injection Attacks via Abstract Syntax Tree-based Neural Network</t>
+          <t>Security of Statistical Databases - Compromise through Attribute Correlational Modeling</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2024</v>
+        <v>1986</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>conf/kbse/2024</t>
+          <t>conf/icde/86</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>db/conf/kbse/ase2024.html#LiX0WZ24</t>
+          <t>db/conf/icde/icde86.html#Palley86</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>@inproceedings{li:2024,
-booktitle = {International Conference on Automated Software Engineering(ASE)}, 
-author = {Yuanlin Li and Zhiwei Xu and Min Zhou 0001 and Hai Wan and Xibin Zhao}, 
-title = {{Trident: Detecting SQL Injection Attacks via Abstract Syntax Tree-based Neural Network}}, 
-year = {2024} 
+          <t>@inproceedings{a.:1986,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Michael A. Palley}, 
+title = {{Security of Statistical Databases - Compromise through Attribute Correlational Modeling}}, 
+year = {1986} 
 }</t>
         </is>
       </c>
@@ -563,44 +563,44 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>conf/kbse/Zhang19</t>
+          <t>conf/icde/HanZFLL22</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>conf/kbse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Kevin Zhang</t>
+          <t>Feng Han and Lan Zhang 0002 and Hanwen Feng 0001 and Weiran Liu and Xiang-Yang Li 0001</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>A Machine Learning Based Approach to Identify SQL Injection Vulnerabilities</t>
+          <t>Scape: Scalable Collaborative Analytics System on Private Database with Malicious Security</t>
         </is>
       </c>
       <c r="E4" t="n">
-        <v>2019</v>
+        <v>2022</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>conf/kbse/2019</t>
+          <t>conf/icde/2022</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>db/conf/kbse/ase2019.html#Zhang19</t>
+          <t>db/conf/icde/icde2022.html#HanZFLL22</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>@inproceedings{zhang:2019,
-booktitle = {International Conference on Automated Software Engineering(ASE)}, 
-author = {Kevin Zhang}, 
-title = {{A Machine Learning Based Approach to Identify SQL Injection Vulnerabilities}}, 
-year = {2019} 
+          <t>@inproceedings{han:2022,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Feng Han and Lan Zhang 0002 and Hanwen Feng 0001 and Weiran Liu and Xiang-Yang Li 0001}, 
+title = {{Scape: Scalable Collaborative Analytics System on Private Database with Malicious Security}}, 
+year = {2022} 
 }</t>
         </is>
       </c>
@@ -608,44 +608,44 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>conf/kbse/ClerissiDMM20</t>
+          <t>conf/icde/Bertino92</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>conf/kbse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Diego Clerissi and Giovanni Denaro and Marco Mobilio and Leonardo Mariani</t>
+          <t>Elisa Bertino</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Plug the Database &amp; Play With Automatic Testing: Improving System Testing by Exploiting Persistent Data</t>
+          <t>Data Hiding and Security in Object-Oriented Databases</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>2020</v>
+        <v>1992</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>conf/kbse/2020</t>
+          <t>conf/icde/92</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>db/conf/kbse/ase2020.html#ClerissiDMM20</t>
+          <t>db/conf/icde/icde92.html#Bertino92</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>@inproceedings{clerissi:2020,
-booktitle = {International Conference on Automated Software Engineering(ASE)}, 
-author = {Diego Clerissi and Giovanni Denaro and Marco Mobilio and Leonardo Mariani}, 
-title = {{Plug the Database &amp; Play With Automatic Testing: Improving System Testing by Exploiting Persistent Data}}, 
-year = {2020} 
+          <t>@inproceedings{bertino:1992,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Elisa Bertino}, 
+title = {{Data Hiding and Security in Object-Oriented Databases}}, 
+year = {1992} 
 }</t>
         </is>
       </c>
@@ -653,44 +653,44 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>conf/kbse/HalfondO05</t>
+          <t>conf/icde/HenningHW87</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>conf/kbse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>William G. J. Halfond and Alessandro Orso</t>
+          <t>Ronda R. Henning and Brian S. Hubbard and Swen A. Walker</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>AMNESIA: analysis and monitoring for NEutralizing SQL-injection attacks</t>
+          <t>Computer Architectures, Database Security, and An Evaluation Metric</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>2005</v>
+        <v>1987</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>conf/kbse/2005</t>
+          <t>conf/icde/87</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>db/conf/kbse/ase2005.html#HalfondO05</t>
+          <t>db/conf/icde/icde87.html#HenningHW87</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>@inproceedings{g.:2005,
-booktitle = {International Conference on Automated Software Engineering(ASE)}, 
-author = {William G. J. Halfond and Alessandro Orso}, 
-title = {{AMNESIA: analysis and monitoring for NEutralizing SQL-injection attacks}}, 
-year = {2005} 
+          <t>@inproceedings{r.:1987,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Ronda R. Henning and Brian S. Hubbard and Swen A. Walker}, 
+title = {{Computer Architectures, Database Security, and An Evaluation Metric}}, 
+year = {1987} 
 }</t>
         </is>
       </c>
@@ -698,22 +698,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>conf/icse/HalfondO06</t>
+          <t>conf/icde/EvdokimovFG06</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>William G. J. Halfond and Alessandro Orso</t>
+          <t>Sergei Evdokimov 0002 and Matthias Fischmann and Oliver Günther 0001</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Preventing SQL injection attacks using AMNESIA</t>
+          <t>Provable Security for Outsourcing Database Operations</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -721,20 +721,20 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>conf/icse/2006</t>
+          <t>conf/icde/2006</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>db/conf/icse/icse2006.html#HalfondO06</t>
+          <t>db/conf/icde/icde2006.html#EvdokimovFG06</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>@inproceedings{g.:2006,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {William G. J. Halfond and Alessandro Orso}, 
-title = {{Preventing SQL injection attacks using AMNESIA}}, 
+          <t>@inproceedings{evdokimov:2006,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Sergei Evdokimov 0002 and Matthias Fischmann and Oliver Günther 0001}, 
+title = {{Provable Security for Outsourcing Database Operations}}, 
 year = {2006} 
 }</t>
         </is>
@@ -743,44 +743,44 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>conf/icse/AbadiFS11</t>
+          <t>conf/icde/JensenKV89</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/icde/</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Aharon Abadi and Yishai A. Feldman and Mati Shomrat</t>
+          <t>Catherine D. Jensen and Robert M. Kiel and Richard D. Verjinski</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Code-motion for API migration: fixing SQL injection vulnerabilities in Java</t>
+          <t>SDDM - A Prototype of a Distributed Architecture for Database Security</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>2011</v>
+        <v>1989</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>conf/icse/2011wrt</t>
+          <t>conf/icde/89</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>db/conf/icse/wrt2011.html#AbadiFS11</t>
+          <t>db/conf/icde/icde89.html#JensenKV89</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>@inproceedings{abadi:2011,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Aharon Abadi and Yishai A. Feldman and Mati Shomrat}, 
-title = {{Code-motion for API migration: fixing SQL injection vulnerabilities in Java}}, 
-year = {2011} 
+          <t>@inproceedings{d.:1989,
+booktitle = {International Conference on Data Engineering (ICDE)}, 
+author = {Catherine D. Jensen and Robert M. Kiel and Richard D. Verjinski}, 
+title = {{SDDM - A Prototype of a Distributed Architecture for Database Security}}, 
+year = {1989} 
 }</t>
         </is>
       </c>
@@ -788,44 +788,44 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>conf/icse/CiampaVP10</t>
+          <t>conf/sigmod/Maurer04</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/sigmod/</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Angelo Ciampa and Corrado Aaron Visaggio and Massimiliano Di Penta</t>
+          <t>Ueli M. Maurer</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>A heuristic-based approach for detecting SQL-injection vulnerabilities in web applications</t>
+          <t>The Role of Cryptography in Database Security</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>2010</v>
+        <v>2004</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>conf/icse/2010sess</t>
+          <t>conf/sigmod/2004</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>db/conf/icse/sess2010.html#CiampaVP10</t>
+          <t>db/conf/sigmod/sigmod2004.html#Maurer04</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>@inproceedings{ciampa:2010,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Angelo Ciampa and Corrado Aaron Visaggio and Massimiliano Di Penta}, 
-title = {{A heuristic-based approach for detecting SQL-injection vulnerabilities in web applications}}, 
-year = {2010} 
+          <t>@inproceedings{m.:2004,
+booktitle = {International Conference on Management of Data (SIGMOD)}, 
+author = {Ueli M. Maurer}, 
+title = {{The Role of Cryptography in Database Security}}, 
+year = {2004} 
 }</t>
         </is>
       </c>
@@ -833,44 +833,44 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>conf/icse/SharT12</t>
+          <t>conf/sigmod/Rosenthal01</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/sigmod/</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Lwin Khin Shar and Hee Beng Kuan Tan</t>
+          <t>Arnon Rosenthal</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Mining input sanitization patterns for predicting SQL injection and cross site scripting vulnerabilities</t>
+          <t>Will Database Researchers Have ANY Role in Data Security? (Panel Abstract)</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>2012</v>
+        <v>2001</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>conf/icse/2012</t>
+          <t>conf/sigmod/2001</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>db/conf/icse/icse2012.html#SharT12</t>
+          <t>db/conf/sigmod/sigmod2001.html#Rosenthal01</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>@inproceedings{khin:2012,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Lwin Khin Shar and Hee Beng Kuan Tan}, 
-title = {{Mining input sanitization patterns for predicting SQL injection and cross site scripting vulnerabilities}}, 
-year = {2012} 
+          <t>@inproceedings{rosenthal:2001,
+booktitle = {International Conference on Management of Data (SIGMOD)}, 
+author = {Arnon Rosenthal}, 
+title = {{Will Database Researchers Have ANY Role in Data Security? (Panel Abstract)}}, 
+year = {2001} 
 }</t>
         </is>
       </c>
@@ -878,44 +878,44 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>conf/icse/KoscinskiHM23</t>
+          <t>conf/sigmod/Morgenstern87</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/sigmod/</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Viktoria Koscinski and Sara Hashemi and Mehdi Mirakhorli</t>
+          <t>Matthew Morgenstern</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>On-Demand Security Requirements Synthesis with Relational Generative Adversarial Networks</t>
+          <t>Security and Inference in Multilevel Database and Knowledge-Base Systems</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>2023</v>
+        <v>1987</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>conf/icse/2023</t>
+          <t>conf/sigmod/87</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>db/conf/icse/icse2023.html#KoscinskiHM23</t>
+          <t>db/conf/sigmod/sigmod87.html#Morgenstern87</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>@inproceedings{koscinski:2023,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Viktoria Koscinski and Sara Hashemi and Mehdi Mirakhorli}, 
-title = {{On-Demand Security Requirements Synthesis with Relational Generative Adversarial Networks}}, 
-year = {2023} 
+          <t>@inproceedings{morgenstern:1987,
+booktitle = {International Conference on Management of Data (SIGMOD)}, 
+author = {Matthew Morgenstern}, 
+title = {{Security and Inference in Multilevel Database and Knowledge-Base Systems}}, 
+year = {1987} 
 }</t>
         </is>
       </c>
@@ -923,44 +923,44 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>conf/icse/KiezunGJE09</t>
+          <t>conf/sigmod/Tajima96</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/sigmod/</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Adam Kiezun and Philip J. Guo and Karthick Jayaraman and Michael D. Ernst</t>
+          <t>Keishi Tajima</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Automatic creation of SQL Injection and cross-site scripting attacks</t>
+          <t>Static Detection of Security Flaws in Object-Oriented Databases</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>2009</v>
+        <v>1996</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>conf/icse/2009</t>
+          <t>conf/sigmod/96</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>db/conf/icse/icse2009.html#KiezunGJE09</t>
+          <t>db/conf/sigmod/sigmod96.html#Tajima96</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>@inproceedings{kiezun:2009,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Adam Kiezun and Philip J. Guo and Karthick Jayaraman and Michael D. Ernst}, 
-title = {{Automatic creation of SQL Injection and cross-site scripting attacks}}, 
-year = {2009} 
+          <t>@inproceedings{tajima:1996,
+booktitle = {International Conference on Management of Data (SIGMOD)}, 
+author = {Keishi Tajima}, 
+title = {{Static Detection of Security Flaws in Object-Oriented Databases}}, 
+year = {1996} 
 }</t>
         </is>
       </c>
@@ -968,44 +968,44 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>conf/icse/PedroC00025</t>
+          <t>conf/sigmod/BenderKG14</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/sigmod/</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Rodrigo Pedro and Miguel E. Coimbra and Daniel Castro 0004 and Paulo Carreira 0001 and Nuno Santos 0001</t>
+          <t>Gabriel Bender and Lucja Kot and Johannes Gehrke</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Prompt-to-SQL Injections in LLM-Integrated Web Applications: Risks and Defenses</t>
+          <t>Explainable security for relational databases</t>
         </is>
       </c>
       <c r="E13" t="n">
-        <v>2025</v>
+        <v>2014</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>conf/icse/2025</t>
+          <t>conf/sigmod/2014</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>db/conf/icse/icse2025.html#PedroC00025</t>
+          <t>db/conf/sigmod/sigmod2014.html#BenderKG14</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>@inproceedings{pedro:2025,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Rodrigo Pedro and Miguel E. Coimbra and Daniel Castro 0004 and Paulo Carreira 0001 and Nuno Santos 0001}, 
-title = {{Prompt-to-SQL Injections in LLM-Integrated Web Applications: Risks and Defenses}}, 
-year = {2025} 
+          <t>@inproceedings{bender:2014,
+booktitle = {International Conference on Management of Data (SIGMOD)}, 
+author = {Gabriel Bender and Lucja Kot and Johannes Gehrke}, 
+title = {{Explainable security for relational databases}}, 
+year = {2014} 
 }</t>
         </is>
       </c>
@@ -1013,44 +1013,44 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>conf/icse/KleinBBWC16</t>
+          <t>conf/sigmod/0001RBMW021</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/sigmod/</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>John Klein and Ross Buglak and David Blockow and Troy Wuttke and Brenton Cooper</t>
+          <t>Xi He 0001 and Jennie Rogers and Johes Bater and Ashwin Machanavajjhala and Chenghong Wang and Xiao Wang 0012</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>A reference architecture for big data systems in the national security domain</t>
+          <t>Practical Security and Privacy for Database Systems</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>2016</v>
+        <v>2021</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>conf/icse/2016bigdse</t>
+          <t>conf/sigmod/2021</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>db/conf/icse/bigdse2016.html#KleinBBWC16</t>
+          <t>db/conf/sigmod/sigmod2021.html#0001RBMW021</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>@inproceedings{klein:2016,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {John Klein and Ross Buglak and David Blockow and Troy Wuttke and Brenton Cooper}, 
-title = {{A reference architecture for big data systems in the national security domain}}, 
-year = {2016} 
+          <t>@inproceedings{he:2021,
+booktitle = {International Conference on Management of Data (SIGMOD)}, 
+author = {Xi He 0001 and Jennie Rogers and Johes Bater and Ashwin Machanavajjhala and Chenghong Wang and Xiao Wang 0012}, 
+title = {{Practical Security and Privacy for Database Systems}}, 
+year = {2021} 
 }</t>
         </is>
       </c>
@@ -1058,44 +1058,44 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>conf/icse/SharTB13</t>
+          <t>conf/vldb/Lockemann78</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/vldb/</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Lwin Khin Shar and Hee Beng Kuan Tan and Lionel C. Briand</t>
+          <t>Peter C. Lockemann</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Mining SQL injection and cross site scripting vulnerabilities using hybrid program analysis</t>
+          <t>Authorization and Database Security</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>2013</v>
+        <v>1978</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>conf/icse/2013</t>
+          <t>conf/vldb/78s</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>db/conf/icse/icse2013.html#SharTB13</t>
+          <t>db/conf/vldb/vldb78s.html#Lockemann78</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>@inproceedings{khin:2013,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Lwin Khin Shar and Hee Beng Kuan Tan and Lionel C. Briand}, 
-title = {{Mining SQL injection and cross site scripting vulnerabilities using hybrid program analysis}}, 
-year = {2013} 
+          <t>@inproceedings{c.:1978,
+booktitle = {International Conference on Very Large Databases (VLDB)}, 
+author = {Peter C. Lockemann}, 
+title = {{Authorization and Database Security}}, 
+year = {1978} 
 }</t>
         </is>
       </c>
@@ -1103,44 +1103,44 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>conf/icse/WeiglUCBV20</t>
+          <t>conf/vldb/DeMillo78</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/vldb/</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alexander Weigl and Mattias Ulbrich and Suhyun Cha and Bernhard Beckert and Birgit Vogel-Heuser</t>
+          <t>Richard A. DeMillo</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Relational Test Tables: A Practical Specification Language for Evolution and Security</t>
+          <t>Database Security</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>2020</v>
+        <v>1978</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>conf/icse/2020formalise</t>
+          <t>conf/vldb/78s</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>db/conf/icse/formalise2020.html#WeiglUCBV20</t>
+          <t>db/conf/vldb/vldb78s.html#DeMillo78</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>@inproceedings{weigl:2020,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Alexander Weigl and Mattias Ulbrich and Suhyun Cha and Bernhard Beckert and Birgit Vogel-Heuser}, 
-title = {{Relational Test Tables: A Practical Specification Language for Evolution and Security}}, 
-year = {2020} 
+          <t>@inproceedings{a.:1978,
+booktitle = {International Conference on Very Large Databases (VLDB)}, 
+author = {Richard A. DeMillo}, 
+title = {{Database Security}}, 
+year = {1978} 
 }</t>
         </is>
       </c>
@@ -1148,44 +1148,44 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>conf/icse/SimosZL19</t>
+          <t>conf/vldb/Davida78a</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>conf/icse/</t>
+          <t>conf/vldb/</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Dimitris E. Simos and Jovan Zivanovic and Manuel Leithner</t>
+          <t>George I. Davida</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Automated combinatorial testing for detecting SQL vulnerabilities in web applications</t>
+          <t>Privacy, Security and Databases: Any Solutions?</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2019</v>
+        <v>1978</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>conf/icse/2019ast</t>
+          <t>conf/vldb/78s</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>db/conf/icse/ast2019.html#SimosZL19</t>
+          <t>db/conf/vldb/vldb78s.html#Davida78a</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>@inproceedings{e.:2019,
-booktitle = {International Conference on Software Engineering (ICSE)}, 
-author = {Dimitris E. Simos and Jovan Zivanovic and Manuel Leithner}, 
-title = {{Automated combinatorial testing for detecting SQL vulnerabilities in web applications}}, 
-year = {2019} 
+          <t>@inproceedings{i.:1978,
+booktitle = {International Conference on Very Large Databases (VLDB)}, 
+author = {George I. Davida}, 
+title = {{Privacy, Security and Databases: Any Solutions?}}, 
+year = {1978} 
 }</t>
         </is>
       </c>
@@ -1193,44 +1193,44 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>conf/sigsoft/HalfondOM06</t>
+          <t>conf/vldb/BussolatiM81</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>conf/sigsoft/</t>
+          <t>conf/vldb/</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>William G. J. Halfond and Alessandro Orso and Panagiotis Manolios</t>
+          <t>U. Bussolati and Giancarlo Martella</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Using positive tainting and syntax-aware evaluation to counter SQL injection attacks</t>
+          <t>A Database Approach to Modelling and Managing Security Information</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>2006</v>
+        <v>1981</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>conf/sigsoft/2006</t>
+          <t>conf/vldb/81</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>db/conf/sigsoft/fse2006.html#HalfondOM06</t>
+          <t>db/conf/vldb/vldb81.html#BussolatiM81</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>@inproceedings{g.:2006,
-booktitle = {Symposium on the Foundations of Software Engineering (FSE)}, 
-author = {William G. J. Halfond and Alessandro Orso and Panagiotis Manolios}, 
-title = {{Using positive tainting and syntax-aware evaluation to counter SQL injection attacks}}, 
-year = {2006} 
+          <t>@inproceedings{bussolati:1981,
+booktitle = {International Conference on Very Large Databases (VLDB)}, 
+author = {U. Bussolati and Giancarlo Martella}, 
+title = {{A Database Approach to Modelling and Managing Security Information}}, 
+year = {1981} 
 }</t>
         </is>
       </c>
@@ -1238,44 +1238,44 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>conf/sigsoft/RamiresRMP25</t>
+          <t>conf/vldb/IdrisGC94</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>conf/sigsoft/</t>
+          <t>conf/vldb/</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Rafael Ramires and Ana Respício and Ibéria Medeiros and Mike Papadakis</t>
+          <t>Norbik Bashah Idris and W. A. Gray and R. F. Churchhouse</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>KAVe: A Tool to Detect XSS and SQLi Vulnerabilities using a Multi-Agent System over a Multi-Layer Knowledge Graph</t>
+          <t>Providing Dynamic Security Control in a Federated Database</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>2025</v>
+        <v>1994</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>conf/sigsoft/2025c</t>
+          <t>conf/vldb/94</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>db/conf/sigsoft/fse2025c.html#RamiresRMP25</t>
+          <t>db/conf/vldb/vldb94.html#IdrisGC94</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>@inproceedings{ramires:2025,
-booktitle = {Symposium on the Foundations of Software Engineering (FSE)}, 
-author = {Rafael Ramires and Ana Respício and Ibéria Medeiros and Mike Papadakis}, 
-title = {{KAVe: A Tool to Detect XSS and SQLi Vulnerabilities using a Multi-Agent System over a Multi-Layer Knowledge Graph}}, 
-year = {2025} 
+          <t>@inproceedings{bashah:1994,
+booktitle = {International Conference on Very Large Databases (VLDB)}, 
+author = {Norbik Bashah Idris and W. A. Gray and R. F. Churchhouse}, 
+title = {{Providing Dynamic Security Control in a Federated Database}}, 
+year = {1994} 
 }</t>
         </is>
       </c>
@@ -1283,44 +1283,40 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>conf/wcre/SiddiqJISI21</t>
+          <t>journals/sigmod/JajodiaS90</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>conf/wcre/</t>
+          <t>journals/sigmod/</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Mohammed Latif Siddiq and Md. Rezwanur Rahman Jahin and Mohammad Rafid Ul Islam and Rifat Shahriyar and Anindya Iqbal</t>
+          <t>Sushil Jajodia and Ravi S. Sandhu</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>SQLIFIX: Learning Based Approach to Fix SQL Injection Vulnerabilities in Source Code</t>
+          <t>Database Security: Current Status and Key Issues</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>2021</v>
-      </c>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>conf/wcre/2021</t>
-        </is>
-      </c>
+        <v>1990</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
       <c r="G20" t="inlineStr">
         <is>
-          <t>db/conf/wcre/saner2021.html#SiddiqJISI21</t>
+          <t>db/journals/sigmod/sigmod19.html#JajodiaS90</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>@inproceedings{latif:2021,
-booktitle = {International Conference on Software Analysis, Evolution and Reengineering (SANER)}, 
-author = {Mohammed Latif Siddiq and Md. Rezwanur Rahman Jahin and Mohammad Rafid Ul Islam and Rifat Shahriyar and Anindya Iqbal}, 
-title = {{SQLIFIX: Learning Based Approach to Fix SQL Injection Vulnerabilities in Source Code}}, 
-year = {2021} 
+          <t>@article{jajodia:1990,
+journal = {SIGMOD Record}, 
+author = {Sushil Jajodia and Ravi S. Sandhu}, 
+title = {{Database Security: Current Status and Key Issues}}, 
+year = {1990} 
 }</t>
         </is>
       </c>
@@ -1328,44 +1324,40 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>conf/wcre/MerloLA06</t>
+          <t>journals/sigmod/PernulL92</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>conf/wcre/</t>
+          <t>journals/sigmod/</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ettore Merlo and Dominic Letarte and Giuliano Antoniol</t>
+          <t>Günther Pernul and Gottfried Luef</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Insider and Ousider Threat-Sensitive SQL Injection Vulnerability Analysis in PHP</t>
+          <t>Bibliography on Database Security</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>2006</v>
-      </c>
-      <c r="F21" t="inlineStr">
-        <is>
-          <t>conf/wcre/2006</t>
-        </is>
-      </c>
+        <v>1992</v>
+      </c>
+      <c r="F21" t="inlineStr"/>
       <c r="G21" t="inlineStr">
         <is>
-          <t>db/conf/wcre/wcre2006.html#MerloLA06</t>
+          <t>db/journals/sigmod/sigmod21.html#PernulL92</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>@inproceedings{merlo:2006,
-booktitle = {International Conference on Software Analysis, Evolution and Reengineering (SANER)}, 
-author = {Ettore Merlo and Dominic Letarte and Giuliano Antoniol}, 
-title = {{Insider and Ousider Threat-Sensitive SQL Injection Vulnerability Analysis in PHP}}, 
-year = {2006} 
+          <t>@article{pernul:1992,
+journal = {SIGMOD Record}, 
+author = {Günther Pernul and Gottfried Luef}, 
+title = {{Bibliography on Database Security}}, 
+year = {1992} 
 }</t>
         </is>
       </c>
@@ -1373,34 +1365,239 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>journals/tse/DavidaLSW78</t>
+          <t>journals/sigmod/NyanchamaO93</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>journals/tse/</t>
+          <t>journals/sigmod/</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>George I. Davida and David J. Linton and C. Russel Szelag and David L. Wells</t>
+          <t>Matunda Nyanchama and Sylvia L. Osborn</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Database Security</t>
+          <t>Role-Based Security, Object Oriented Databases &amp; Separation of Duty</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>1978</v>
+        <v>1993</v>
       </c>
       <c r="F22" t="inlineStr"/>
       <c r="G22" t="inlineStr">
         <is>
+          <t>db/journals/sigmod/sigmod22.html#NyanchamaO93</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>@article{nyanchama:1993,
+journal = {SIGMOD Record}, 
+author = {Matunda Nyanchama and Sylvia L. Osborn}, 
+title = {{Role-Based Security, Object Oriented Databases &amp; Separation of Duty}}, 
+year = {1993} 
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>journals/sigmod/LuntF90</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>journals/sigmod/</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Teresa F. Lunt and Eduardo B. Fernández</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Database Security</t>
+        </is>
+      </c>
+      <c r="E23" t="n">
+        <v>1990</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>db/journals/sigmod/sigmod19.html#LuntF90</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>@article{f.:1990,
+journal = {SIGMOD Record}, 
+author = {Teresa F. Lunt and Eduardo B. Fernández}, 
+title = {{Database Security}}, 
+year = {1990} 
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>journals/is/Michalewicz87</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>journals/is/</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Zbigniew Michalewicz</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Functional dependencies and their connection with security of statistical databases</t>
+        </is>
+      </c>
+      <c r="E24" t="n">
+        <v>1987</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>db/journals/is/is12.html#Michalewicz87</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>@article{michalewicz:1987,
+journal = {Information Systems}, 
+author = {Zbigniew Michalewicz}, 
+title = {{Functional dependencies and their connection with security of statistical databases}}, 
+year = {1987} 
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>journals/is/BertinoJS95</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>journals/is/</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Elisa Bertino and Sushil Jajodia and Pierangela Samarati</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Database Security: Research and Practice</t>
+        </is>
+      </c>
+      <c r="E25" t="n">
+        <v>1995</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>db/journals/is/is20.html#BertinoJS95</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>@article{bertino:1995,
+journal = {Information Systems}, 
+author = {Elisa Bertino and Sushil Jajodia and Pierangela Samarati}, 
+title = {{Database Security: Research and Practice}}, 
+year = {1995} 
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>journals/is/Hartson81</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>journals/is/</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>H. Rex Hartson</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Database security-system architectures</t>
+        </is>
+      </c>
+      <c r="E26" t="n">
+        <v>1981</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>db/journals/is/is6.html#Hartson81</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>@article{rex:1981,
+journal = {Information Systems}, 
+author = {H. Rex Hartson}, 
+title = {{Database security-system architectures}}, 
+year = {1981} 
+}</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>journals/tse/DavidaLSW78</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>journals/tse/</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>George I. Davida and David J. Linton and C. Russel Szelag and David L. Wells</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Database Security</t>
+        </is>
+      </c>
+      <c r="E27" t="n">
+        <v>1978</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
           <t>db/journals/tse/tse4.html#DavidaLSW78</t>
         </is>
       </c>
-      <c r="H22" t="inlineStr">
+      <c r="H27" t="inlineStr">
         <is>
           <t>@article{i.:1978,
 journal = {Transactions on Software Engineering (TSE)}, 
@@ -1411,37 +1608,37 @@
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>journals/tse/DenningAHLMNS87</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>journals/tse/</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>Dorothy E. Denning and Selim G. Akl and Mark R. Heckman and Teresa F. Lunt and Matthew Morgenstern and Peter G. Neumann and Roger R. Schell</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr">
+      <c r="D28" t="inlineStr">
         <is>
           <t>Views for Multilevel Database Security</t>
         </is>
       </c>
-      <c r="E23" t="n">
+      <c r="E28" t="n">
         <v>1987</v>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr">
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr">
         <is>
           <t>db/journals/tse/tse13.html#DenningAHLMNS87</t>
         </is>
       </c>
-      <c r="H23" t="inlineStr">
+      <c r="H28" t="inlineStr">
         <is>
           <t>@article{e.:1987,
 journal = {Transactions on Software Engineering (TSE)}, 
@@ -1452,37 +1649,37 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
+    <row r="29">
+      <c r="A29" t="inlineStr">
         <is>
           <t>journals/tse/OzsoyogluC82</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B29" t="inlineStr">
         <is>
           <t>journals/tse/</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>Gultekin Özsoyoglu and Francis Y. L. Chin</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D29" t="inlineStr">
         <is>
           <t>Enhancing the Security of Statistical Databases with a Question-Answering System and a Kernel Design</t>
         </is>
       </c>
-      <c r="E24" t="n">
+      <c r="E29" t="n">
         <v>1982</v>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr">
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr">
         <is>
           <t>db/journals/tse/tse8.html#OzsoyogluC82</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H29" t="inlineStr">
         <is>
           <t>@article{özsoyoglu:1982,
 journal = {Transactions on Software Engineering (TSE)}, 

</xml_diff>